<commit_message>
자료 업뎃, minor update
</commit_message>
<xml_diff>
--- a/X-Series/XD04P/LED_Module_Control_BD/XD04_LED_Module_Control_BD/Docs/xdic_led_module_info.xlsx
+++ b/X-Series/XD04P/LED_Module_Control_BD/XD04_LED_Module_Control_BD/Docs/xdic_led_module_info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\X-Series\XD04P\LED_Module_Control_BD\XD04_LED_Module_Control_BD\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D785DF4-F663-4DE0-98DF-27DF7E26A03D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3256A65-BFEA-4D43-B402-BF7FE6B8567C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43080" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="protocol" sheetId="1" r:id="rId1"/>
@@ -1653,7 +1653,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="130">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1958,91 +1958,88 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3848,14 +3845,14 @@
       <c r="D7" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="103" t="s">
+      <c r="E7" s="109" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="103"/>
-      <c r="G7" s="103"/>
-      <c r="H7" s="103"/>
-      <c r="I7" s="103"/>
-      <c r="J7" s="103"/>
+      <c r="F7" s="109"/>
+      <c r="G7" s="109"/>
+      <c r="H7" s="109"/>
+      <c r="I7" s="109"/>
+      <c r="J7" s="109"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B8" s="2" t="s">
@@ -3867,14 +3864,14 @@
       <c r="D8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="102" t="s">
+      <c r="E8" s="110" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="102"/>
-      <c r="G8" s="102"/>
-      <c r="H8" s="102"/>
-      <c r="I8" s="102"/>
-      <c r="J8" s="102"/>
+      <c r="F8" s="110"/>
+      <c r="G8" s="110"/>
+      <c r="H8" s="110"/>
+      <c r="I8" s="110"/>
+      <c r="J8" s="110"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B9" s="2" t="s">
@@ -3905,14 +3902,14 @@
       <c r="D10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="102" t="s">
+      <c r="E10" s="110" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="102"/>
-      <c r="G10" s="102"/>
-      <c r="H10" s="102"/>
-      <c r="I10" s="102"/>
-      <c r="J10" s="102"/>
+      <c r="F10" s="110"/>
+      <c r="G10" s="110"/>
+      <c r="H10" s="110"/>
+      <c r="I10" s="110"/>
+      <c r="J10" s="110"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B11" s="2" t="s">
@@ -3943,14 +3940,14 @@
       <c r="D12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="102" t="s">
+      <c r="E12" s="110" t="s">
         <v>63</v>
       </c>
-      <c r="F12" s="102"/>
-      <c r="G12" s="102"/>
-      <c r="H12" s="102"/>
-      <c r="I12" s="102"/>
-      <c r="J12" s="102"/>
+      <c r="F12" s="110"/>
+      <c r="G12" s="110"/>
+      <c r="H12" s="110"/>
+      <c r="I12" s="110"/>
+      <c r="J12" s="110"/>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B13" s="2" t="s">
@@ -3989,13 +3986,13 @@
       <c r="E17" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F17" s="103" t="s">
+      <c r="F17" s="109" t="s">
         <v>54</v>
       </c>
-      <c r="G17" s="103"/>
-      <c r="H17" s="103"/>
-      <c r="I17" s="103"/>
-      <c r="J17" s="103"/>
+      <c r="G17" s="109"/>
+      <c r="H17" s="109"/>
+      <c r="I17" s="109"/>
+      <c r="J17" s="109"/>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B18" s="3" t="s">
@@ -4010,13 +4007,13 @@
       <c r="E18" s="4">
         <v>0</v>
       </c>
-      <c r="F18" s="102" t="s">
+      <c r="F18" s="110" t="s">
         <v>203</v>
       </c>
-      <c r="G18" s="102"/>
-      <c r="H18" s="102"/>
-      <c r="I18" s="102"/>
-      <c r="J18" s="102"/>
+      <c r="G18" s="110"/>
+      <c r="H18" s="110"/>
+      <c r="I18" s="110"/>
+      <c r="J18" s="110"/>
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B19" s="3" t="s">
@@ -4031,13 +4028,13 @@
       <c r="E19" s="4">
         <v>0</v>
       </c>
-      <c r="F19" s="102" t="s">
+      <c r="F19" s="110" t="s">
         <v>198</v>
       </c>
-      <c r="G19" s="102"/>
-      <c r="H19" s="102"/>
-      <c r="I19" s="102"/>
-      <c r="J19" s="102"/>
+      <c r="G19" s="110"/>
+      <c r="H19" s="110"/>
+      <c r="I19" s="110"/>
+      <c r="J19" s="110"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B20" s="3" t="s">
@@ -4052,13 +4049,13 @@
       <c r="E20" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="F20" s="102" t="s">
+      <c r="F20" s="110" t="s">
         <v>119</v>
       </c>
-      <c r="G20" s="102"/>
-      <c r="H20" s="102"/>
-      <c r="I20" s="102"/>
-      <c r="J20" s="102"/>
+      <c r="G20" s="110"/>
+      <c r="H20" s="110"/>
+      <c r="I20" s="110"/>
+      <c r="J20" s="110"/>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B21" s="3" t="s">
@@ -4073,13 +4070,13 @@
       <c r="E21" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="F21" s="126" t="s">
+      <c r="F21" s="129" t="s">
         <v>229</v>
       </c>
-      <c r="G21" s="126"/>
-      <c r="H21" s="126"/>
-      <c r="I21" s="126"/>
-      <c r="J21" s="126"/>
+      <c r="G21" s="129"/>
+      <c r="H21" s="129"/>
+      <c r="I21" s="129"/>
+      <c r="J21" s="129"/>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B22" s="3" t="s">
@@ -4094,13 +4091,13 @@
       <c r="E22" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F22" s="102" t="s">
+      <c r="F22" s="110" t="s">
         <v>215</v>
       </c>
-      <c r="G22" s="102"/>
-      <c r="H22" s="102"/>
-      <c r="I22" s="102"/>
-      <c r="J22" s="102"/>
+      <c r="G22" s="110"/>
+      <c r="H22" s="110"/>
+      <c r="I22" s="110"/>
+      <c r="J22" s="110"/>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B23" s="3" t="s">
@@ -4115,13 +4112,13 @@
       <c r="E23" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="102" t="s">
+      <c r="F23" s="110" t="s">
         <v>216</v>
       </c>
-      <c r="G23" s="102"/>
-      <c r="H23" s="102"/>
-      <c r="I23" s="102"/>
-      <c r="J23" s="102"/>
+      <c r="G23" s="110"/>
+      <c r="H23" s="110"/>
+      <c r="I23" s="110"/>
+      <c r="J23" s="110"/>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B24" s="3" t="s">
@@ -4136,13 +4133,13 @@
       <c r="E24" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="F24" s="102" t="s">
+      <c r="F24" s="110" t="s">
         <v>217</v>
       </c>
-      <c r="G24" s="102"/>
-      <c r="H24" s="102"/>
-      <c r="I24" s="102"/>
-      <c r="J24" s="102"/>
+      <c r="G24" s="110"/>
+      <c r="H24" s="110"/>
+      <c r="I24" s="110"/>
+      <c r="J24" s="110"/>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B25" s="3" t="s">
@@ -4157,13 +4154,13 @@
       <c r="E25" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="F25" s="102" t="s">
+      <c r="F25" s="110" t="s">
         <v>218</v>
       </c>
-      <c r="G25" s="102"/>
-      <c r="H25" s="102"/>
-      <c r="I25" s="102"/>
-      <c r="J25" s="102"/>
+      <c r="G25" s="110"/>
+      <c r="H25" s="110"/>
+      <c r="I25" s="110"/>
+      <c r="J25" s="110"/>
       <c r="L25" s="101" t="s">
         <v>221</v>
       </c>
@@ -4193,63 +4190,52 @@
       <c r="E26" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="F26" s="102" t="s">
+      <c r="F26" s="110" t="s">
         <v>220</v>
       </c>
-      <c r="G26" s="102"/>
-      <c r="H26" s="102"/>
-      <c r="I26" s="102"/>
-      <c r="J26" s="102"/>
+      <c r="G26" s="110"/>
+      <c r="H26" s="110"/>
+      <c r="I26" s="110"/>
+      <c r="J26" s="110"/>
       <c r="L26" s="6">
         <v>800</v>
       </c>
-      <c r="M26" s="128">
+      <c r="M26" s="103">
         <f>L26/4095*128</f>
         <v>25.006105006105006</v>
       </c>
-      <c r="N26" s="129">
+      <c r="N26" s="6">
         <v>20</v>
       </c>
-      <c r="O26" s="130">
+      <c r="O26" s="104">
         <f>N26/16383</f>
         <v>1.2207776353537203E-3</v>
       </c>
-      <c r="P26" s="128">
+      <c r="P26" s="103">
         <f>M26*O26</f>
         <v>3.0526893738759699E-2</v>
       </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B27" s="127" t="s">
+      <c r="B27" s="102" t="s">
         <v>226</v>
       </c>
-      <c r="C27" s="127" t="s">
+      <c r="C27" s="102" t="s">
         <v>227</v>
       </c>
-      <c r="D27" s="127" t="s">
+      <c r="D27" s="102" t="s">
         <v>5</v>
       </c>
-      <c r="E27" s="127" t="s">
+      <c r="E27" s="102" t="s">
         <v>228</v>
       </c>
-      <c r="F27" s="126" t="s">
+      <c r="F27" s="112" t="s">
         <v>230</v>
       </c>
-      <c r="G27" s="126"/>
-      <c r="H27" s="126"/>
-      <c r="I27" s="126"/>
-      <c r="J27" s="126"/>
-    </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B28" s="125"/>
-      <c r="C28" s="125"/>
-      <c r="D28" s="125"/>
-      <c r="E28" s="125"/>
-      <c r="F28" s="125"/>
-      <c r="G28" s="125"/>
-      <c r="H28" s="125"/>
-      <c r="I28" s="125"/>
-      <c r="J28" s="125"/>
+      <c r="G27" s="112"/>
+      <c r="H27" s="112"/>
+      <c r="I27" s="112"/>
+      <c r="J27" s="112"/>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B30" s="5" t="s">
@@ -4265,16 +4251,16 @@
         <v>47</v>
       </c>
       <c r="E31" s="10"/>
-      <c r="F31" s="104" t="s">
+      <c r="F31" s="111" t="s">
         <v>47</v>
       </c>
-      <c r="G31" s="104"/>
-      <c r="H31" s="104"/>
-      <c r="I31" s="104"/>
-      <c r="J31" s="104"/>
-      <c r="K31" s="104"/>
-      <c r="L31" s="104"/>
-      <c r="M31" s="104"/>
+      <c r="G31" s="111"/>
+      <c r="H31" s="111"/>
+      <c r="I31" s="111"/>
+      <c r="J31" s="111"/>
+      <c r="K31" s="111"/>
+      <c r="L31" s="111"/>
+      <c r="M31" s="111"/>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B32" s="8" t="s">
@@ -4541,11 +4527,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="E9:J9"/>
-    <mergeCell ref="E11:J11"/>
-    <mergeCell ref="E13:J13"/>
-    <mergeCell ref="F17:J17"/>
     <mergeCell ref="F25:J25"/>
     <mergeCell ref="E7:J7"/>
     <mergeCell ref="F31:M31"/>
@@ -4561,6 +4542,11 @@
     <mergeCell ref="F20:J20"/>
     <mergeCell ref="F26:J26"/>
     <mergeCell ref="F27:J27"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="E9:J9"/>
+    <mergeCell ref="E11:J11"/>
+    <mergeCell ref="E13:J13"/>
+    <mergeCell ref="F17:J17"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4580,28 +4566,28 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="109" t="s">
+      <c r="B2" s="113" t="s">
         <v>105</v>
       </c>
-      <c r="D2" s="104" t="s">
+      <c r="D2" s="111" t="s">
         <v>84</v>
       </c>
-      <c r="E2" s="104" t="s">
+      <c r="E2" s="111" t="s">
         <v>72</v>
       </c>
-      <c r="F2" s="104"/>
-      <c r="G2" s="104"/>
-      <c r="H2" s="104"/>
-      <c r="I2" s="104" t="s">
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111" t="s">
         <v>71</v>
       </c>
-      <c r="J2" s="104"/>
-      <c r="K2" s="104"/>
-      <c r="L2" s="104"/>
+      <c r="J2" s="111"/>
+      <c r="K2" s="111"/>
+      <c r="L2" s="111"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B3" s="110"/>
-      <c r="D3" s="104"/>
+      <c r="B3" s="114"/>
+      <c r="D3" s="111"/>
       <c r="E3" s="7" t="s">
         <v>112</v>
       </c>
@@ -5783,35 +5769,35 @@
       </c>
     </row>
     <row r="3" spans="2:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="114" t="s">
+      <c r="B3" s="118" t="s">
         <v>169</v>
       </c>
-      <c r="C3" s="117" t="s">
+      <c r="C3" s="121" t="s">
         <v>171</v>
       </c>
-      <c r="D3" s="118" t="s">
+      <c r="D3" s="123" t="s">
         <v>172</v>
       </c>
-      <c r="F3" s="114" t="s">
+      <c r="F3" s="118" t="s">
         <v>72</v>
       </c>
-      <c r="G3" s="117"/>
-      <c r="H3" s="117"/>
-      <c r="I3" s="117"/>
-      <c r="J3" s="117" t="s">
+      <c r="G3" s="121"/>
+      <c r="H3" s="121"/>
+      <c r="I3" s="121"/>
+      <c r="J3" s="121" t="s">
         <v>71</v>
       </c>
-      <c r="K3" s="117"/>
-      <c r="L3" s="117"/>
-      <c r="M3" s="121"/>
-      <c r="N3" s="111" t="s">
+      <c r="K3" s="121"/>
+      <c r="L3" s="121"/>
+      <c r="M3" s="126"/>
+      <c r="N3" s="115" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.45">
-      <c r="B4" s="115"/>
-      <c r="C4" s="104"/>
-      <c r="D4" s="119"/>
+      <c r="B4" s="119"/>
+      <c r="C4" s="111"/>
+      <c r="D4" s="124"/>
       <c r="F4" s="60" t="s">
         <v>112</v>
       </c>
@@ -5836,12 +5822,12 @@
       <c r="M4" s="72" t="s">
         <v>115</v>
       </c>
-      <c r="N4" s="112"/>
+      <c r="N4" s="116"/>
     </row>
     <row r="5" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B5" s="122"/>
-      <c r="C5" s="123"/>
-      <c r="D5" s="124"/>
+      <c r="B5" s="120"/>
+      <c r="C5" s="122"/>
+      <c r="D5" s="125"/>
       <c r="F5" s="70">
         <v>1</v>
       </c>
@@ -5873,7 +5859,7 @@
         <f t="shared" si="0"/>
         <v>141</v>
       </c>
-      <c r="N5" s="113"/>
+      <c r="N5" s="117"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B6" s="66">
@@ -6261,35 +6247,35 @@
       </c>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.45">
-      <c r="B19" s="114" t="s">
+      <c r="B19" s="118" t="s">
         <v>169</v>
       </c>
-      <c r="C19" s="117" t="s">
+      <c r="C19" s="121" t="s">
         <v>171</v>
       </c>
-      <c r="D19" s="118" t="s">
+      <c r="D19" s="123" t="s">
         <v>172</v>
       </c>
-      <c r="F19" s="114" t="s">
+      <c r="F19" s="118" t="s">
         <v>72</v>
       </c>
-      <c r="G19" s="117"/>
-      <c r="H19" s="117"/>
-      <c r="I19" s="117"/>
-      <c r="J19" s="117" t="s">
+      <c r="G19" s="121"/>
+      <c r="H19" s="121"/>
+      <c r="I19" s="121"/>
+      <c r="J19" s="121" t="s">
         <v>71</v>
       </c>
-      <c r="K19" s="117"/>
-      <c r="L19" s="117"/>
-      <c r="M19" s="121"/>
-      <c r="N19" s="111" t="s">
+      <c r="K19" s="121"/>
+      <c r="L19" s="121"/>
+      <c r="M19" s="126"/>
+      <c r="N19" s="115" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.45">
-      <c r="B20" s="115"/>
-      <c r="C20" s="104"/>
-      <c r="D20" s="119"/>
+      <c r="B20" s="119"/>
+      <c r="C20" s="111"/>
+      <c r="D20" s="124"/>
       <c r="F20" s="60" t="s">
         <v>112</v>
       </c>
@@ -6314,12 +6300,12 @@
       <c r="M20" s="72" t="s">
         <v>115</v>
       </c>
-      <c r="N20" s="112"/>
+      <c r="N20" s="116"/>
     </row>
     <row r="21" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B21" s="116"/>
-      <c r="C21" s="109"/>
-      <c r="D21" s="120"/>
+      <c r="B21" s="127"/>
+      <c r="C21" s="113"/>
+      <c r="D21" s="128"/>
       <c r="F21" s="90">
         <v>12</v>
       </c>
@@ -6351,7 +6337,7 @@
         <f t="shared" ref="M21" si="7">L21+20</f>
         <v>152</v>
       </c>
-      <c r="N21" s="113"/>
+      <c r="N21" s="117"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B22" s="85">
@@ -6849,18 +6835,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="N19:N21"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="D19:D21"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="J19:M19"/>
     <mergeCell ref="N3:N5"/>
     <mergeCell ref="B3:B5"/>
     <mergeCell ref="C3:C5"/>
     <mergeCell ref="D3:D5"/>
     <mergeCell ref="F3:I3"/>
     <mergeCell ref="J3:M3"/>
-    <mergeCell ref="N19:N21"/>
-    <mergeCell ref="B19:B21"/>
-    <mergeCell ref="C19:C21"/>
-    <mergeCell ref="D19:D21"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="J19:M19"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
daisy 갯수 입력 가능(default daisy 2개)
</commit_message>
<xml_diff>
--- a/X-Series/XD04P/LED_Module_Control_BD/XD04_LED_Module_Control_BD/Docs/xdic_led_module_info.xlsx
+++ b/X-Series/XD04P/LED_Module_Control_BD/XD04_LED_Module_Control_BD/Docs/xdic_led_module_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\X-Series\XD04P\LED_Module_Control_BD\XD04_LED_Module_Control_BD\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3256A65-BFEA-4D43-B402-BF7FE6B8567C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB83A3E-0ED7-4B87-A894-B0C5BFCDAA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="protocol" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="235">
   <si>
     <t>SOP</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -900,10 +900,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Baudrate = 115200, Parity = None, Stopbits = 1-bit, Data = 8-bits, Protocol 사이 10ms delay 필요</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Duty</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -921,6 +917,26 @@
   </si>
   <si>
     <t>LED 전류 Duty 설정 (1% 단위 조절)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Model Select</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x08</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1 or 2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1 : Model for one XD04, 2 : Model for two XD04s</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Baudrate = 115200, Parity = None, Stopbits = 1-bit, Data = 8-bits, Protocol 사이 최소 10ms delay 필요</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1653,7 +1669,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="134">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1967,6 +1983,15 @@
     <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1979,65 +2004,68 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2077,14 +2105,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>75</xdr:row>
-      <xdr:rowOff>28258</xdr:rowOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>31432</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2127,7 +2155,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>54</xdr:row>
+      <xdr:row>55</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="572849" cy="280205"/>
@@ -2198,7 +2226,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>352425</xdr:colOff>
-      <xdr:row>66</xdr:row>
+      <xdr:row>67</xdr:row>
       <xdr:rowOff>161925</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="497059" cy="280205"/>
@@ -2271,14 +2299,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>78</xdr:row>
+      <xdr:row>79</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>107</xdr:row>
-      <xdr:rowOff>28258</xdr:rowOff>
+      <xdr:row>108</xdr:row>
+      <xdr:rowOff>31433</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2321,7 +2349,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>247650</xdr:colOff>
-      <xdr:row>86</xdr:row>
+      <xdr:row>87</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="572849" cy="280205"/>
@@ -2392,7 +2420,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>361950</xdr:colOff>
-      <xdr:row>99</xdr:row>
+      <xdr:row>100</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="497059" cy="280205"/>
@@ -2465,13 +2493,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>95</xdr:row>
+      <xdr:row>96</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>514350</xdr:colOff>
-      <xdr:row>95</xdr:row>
+      <xdr:row>96</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -2522,13 +2550,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>542925</xdr:colOff>
-      <xdr:row>95</xdr:row>
+      <xdr:row>96</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>1590675</xdr:colOff>
-      <xdr:row>95</xdr:row>
+      <xdr:row>96</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -2579,7 +2607,7 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>504825</xdr:colOff>
-      <xdr:row>93</xdr:row>
+      <xdr:row>94</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="701282" cy="436786"/>
@@ -2662,7 +2690,7 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>537156</xdr:colOff>
-      <xdr:row>92</xdr:row>
+      <xdr:row>93</xdr:row>
       <xdr:rowOff>161925</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1093826" cy="436786"/>
@@ -2745,14 +2773,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>110</xdr:row>
+      <xdr:row>111</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>685800</xdr:colOff>
-      <xdr:row>139</xdr:row>
-      <xdr:rowOff>28256</xdr:rowOff>
+      <xdr:row>140</xdr:row>
+      <xdr:rowOff>31431</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2795,7 +2823,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>238125</xdr:colOff>
-      <xdr:row>118</xdr:row>
+      <xdr:row>119</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="572849" cy="280205"/>
@@ -2866,7 +2894,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>352425</xdr:colOff>
-      <xdr:row>130</xdr:row>
+      <xdr:row>131</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="497059" cy="280205"/>
@@ -2939,13 +2967,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>295275</xdr:colOff>
-      <xdr:row>127</xdr:row>
+      <xdr:row>128</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>504825</xdr:colOff>
-      <xdr:row>127</xdr:row>
+      <xdr:row>128</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -2996,13 +3024,13 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>127</xdr:row>
+      <xdr:row>128</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
       <xdr:colOff>1581150</xdr:colOff>
-      <xdr:row>127</xdr:row>
+      <xdr:row>128</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -3053,7 +3081,7 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>495300</xdr:colOff>
-      <xdr:row>124</xdr:row>
+      <xdr:row>125</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="701282" cy="436786"/>
@@ -3136,7 +3164,7 @@
     <xdr:from>
       <xdr:col>5</xdr:col>
       <xdr:colOff>527629</xdr:colOff>
-      <xdr:row>124</xdr:row>
+      <xdr:row>125</xdr:row>
       <xdr:rowOff>104775</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1093826" cy="436786"/>
@@ -3764,7 +3792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:P110"/>
+  <dimension ref="B2:P111"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.58203125" style="6" customWidth="1"/>
@@ -3786,14 +3814,14 @@
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B3" s="105" t="s">
-        <v>225</v>
-      </c>
-      <c r="C3" s="105"/>
-      <c r="D3" s="105"/>
-      <c r="E3" s="105"/>
-      <c r="F3" s="105"/>
-      <c r="G3" s="105"/>
+      <c r="B3" s="108" t="s">
+        <v>234</v>
+      </c>
+      <c r="C3" s="108"/>
+      <c r="D3" s="108"/>
+      <c r="E3" s="108"/>
+      <c r="F3" s="108"/>
+      <c r="G3" s="108"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B4" s="1" t="s">
@@ -3845,14 +3873,14 @@
       <c r="D7" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="109" t="s">
+      <c r="E7" s="106" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="109"/>
-      <c r="G7" s="109"/>
-      <c r="H7" s="109"/>
-      <c r="I7" s="109"/>
-      <c r="J7" s="109"/>
+      <c r="F7" s="106"/>
+      <c r="G7" s="106"/>
+      <c r="H7" s="106"/>
+      <c r="I7" s="106"/>
+      <c r="J7" s="106"/>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B8" s="2" t="s">
@@ -3864,14 +3892,14 @@
       <c r="D8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="110" t="s">
+      <c r="E8" s="105" t="s">
         <v>65</v>
       </c>
-      <c r="F8" s="110"/>
-      <c r="G8" s="110"/>
-      <c r="H8" s="110"/>
-      <c r="I8" s="110"/>
-      <c r="J8" s="110"/>
+      <c r="F8" s="105"/>
+      <c r="G8" s="105"/>
+      <c r="H8" s="105"/>
+      <c r="I8" s="105"/>
+      <c r="J8" s="105"/>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B9" s="2" t="s">
@@ -3883,14 +3911,14 @@
       <c r="D9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="106" t="s">
+      <c r="E9" s="109" t="s">
         <v>168</v>
       </c>
-      <c r="F9" s="107"/>
-      <c r="G9" s="107"/>
-      <c r="H9" s="107"/>
-      <c r="I9" s="107"/>
-      <c r="J9" s="108"/>
+      <c r="F9" s="110"/>
+      <c r="G9" s="110"/>
+      <c r="H9" s="110"/>
+      <c r="I9" s="110"/>
+      <c r="J9" s="111"/>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B10" s="2" t="s">
@@ -3902,14 +3930,14 @@
       <c r="D10" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="110" t="s">
+      <c r="E10" s="105" t="s">
         <v>69</v>
       </c>
-      <c r="F10" s="110"/>
-      <c r="G10" s="110"/>
-      <c r="H10" s="110"/>
-      <c r="I10" s="110"/>
-      <c r="J10" s="110"/>
+      <c r="F10" s="105"/>
+      <c r="G10" s="105"/>
+      <c r="H10" s="105"/>
+      <c r="I10" s="105"/>
+      <c r="J10" s="105"/>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B11" s="2" t="s">
@@ -3921,14 +3949,14 @@
       <c r="D11" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="106" t="s">
+      <c r="E11" s="109" t="s">
         <v>214</v>
       </c>
-      <c r="F11" s="107"/>
-      <c r="G11" s="107"/>
-      <c r="H11" s="107"/>
-      <c r="I11" s="107"/>
-      <c r="J11" s="108"/>
+      <c r="F11" s="110"/>
+      <c r="G11" s="110"/>
+      <c r="H11" s="110"/>
+      <c r="I11" s="110"/>
+      <c r="J11" s="111"/>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B12" s="2" t="s">
@@ -3940,14 +3968,14 @@
       <c r="D12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="110" t="s">
+      <c r="E12" s="105" t="s">
         <v>63</v>
       </c>
-      <c r="F12" s="110"/>
-      <c r="G12" s="110"/>
-      <c r="H12" s="110"/>
-      <c r="I12" s="110"/>
-      <c r="J12" s="110"/>
+      <c r="F12" s="105"/>
+      <c r="G12" s="105"/>
+      <c r="H12" s="105"/>
+      <c r="I12" s="105"/>
+      <c r="J12" s="105"/>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B13" s="2" t="s">
@@ -3959,14 +3987,14 @@
       <c r="D13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="106" t="s">
+      <c r="E13" s="109" t="s">
         <v>64</v>
       </c>
-      <c r="F13" s="107"/>
-      <c r="G13" s="107"/>
-      <c r="H13" s="107"/>
-      <c r="I13" s="107"/>
-      <c r="J13" s="108"/>
+      <c r="F13" s="110"/>
+      <c r="G13" s="110"/>
+      <c r="H13" s="110"/>
+      <c r="I13" s="110"/>
+      <c r="J13" s="111"/>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B16" s="5" t="s">
@@ -3986,13 +4014,13 @@
       <c r="E17" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F17" s="109" t="s">
+      <c r="F17" s="106" t="s">
         <v>54</v>
       </c>
-      <c r="G17" s="109"/>
-      <c r="H17" s="109"/>
-      <c r="I17" s="109"/>
-      <c r="J17" s="109"/>
+      <c r="G17" s="106"/>
+      <c r="H17" s="106"/>
+      <c r="I17" s="106"/>
+      <c r="J17" s="106"/>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B18" s="3" t="s">
@@ -4007,13 +4035,13 @@
       <c r="E18" s="4">
         <v>0</v>
       </c>
-      <c r="F18" s="110" t="s">
+      <c r="F18" s="105" t="s">
         <v>203</v>
       </c>
-      <c r="G18" s="110"/>
-      <c r="H18" s="110"/>
-      <c r="I18" s="110"/>
-      <c r="J18" s="110"/>
+      <c r="G18" s="105"/>
+      <c r="H18" s="105"/>
+      <c r="I18" s="105"/>
+      <c r="J18" s="105"/>
     </row>
     <row r="19" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B19" s="3" t="s">
@@ -4028,13 +4056,13 @@
       <c r="E19" s="4">
         <v>0</v>
       </c>
-      <c r="F19" s="110" t="s">
+      <c r="F19" s="105" t="s">
         <v>198</v>
       </c>
-      <c r="G19" s="110"/>
-      <c r="H19" s="110"/>
-      <c r="I19" s="110"/>
-      <c r="J19" s="110"/>
+      <c r="G19" s="105"/>
+      <c r="H19" s="105"/>
+      <c r="I19" s="105"/>
+      <c r="J19" s="105"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B20" s="3" t="s">
@@ -4049,13 +4077,13 @@
       <c r="E20" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="F20" s="110" t="s">
+      <c r="F20" s="105" t="s">
         <v>119</v>
       </c>
-      <c r="G20" s="110"/>
-      <c r="H20" s="110"/>
-      <c r="I20" s="110"/>
-      <c r="J20" s="110"/>
+      <c r="G20" s="105"/>
+      <c r="H20" s="105"/>
+      <c r="I20" s="105"/>
+      <c r="J20" s="105"/>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B21" s="3" t="s">
@@ -4070,13 +4098,13 @@
       <c r="E21" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="F21" s="129" t="s">
-        <v>229</v>
-      </c>
-      <c r="G21" s="129"/>
-      <c r="H21" s="129"/>
-      <c r="I21" s="129"/>
-      <c r="J21" s="129"/>
+      <c r="F21" s="105" t="s">
+        <v>228</v>
+      </c>
+      <c r="G21" s="105"/>
+      <c r="H21" s="105"/>
+      <c r="I21" s="105"/>
+      <c r="J21" s="105"/>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B22" s="3" t="s">
@@ -4091,13 +4119,13 @@
       <c r="E22" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F22" s="110" t="s">
+      <c r="F22" s="105" t="s">
         <v>215</v>
       </c>
-      <c r="G22" s="110"/>
-      <c r="H22" s="110"/>
-      <c r="I22" s="110"/>
-      <c r="J22" s="110"/>
+      <c r="G22" s="105"/>
+      <c r="H22" s="105"/>
+      <c r="I22" s="105"/>
+      <c r="J22" s="105"/>
     </row>
     <row r="23" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B23" s="3" t="s">
@@ -4112,13 +4140,13 @@
       <c r="E23" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F23" s="110" t="s">
+      <c r="F23" s="105" t="s">
         <v>216</v>
       </c>
-      <c r="G23" s="110"/>
-      <c r="H23" s="110"/>
-      <c r="I23" s="110"/>
-      <c r="J23" s="110"/>
+      <c r="G23" s="105"/>
+      <c r="H23" s="105"/>
+      <c r="I23" s="105"/>
+      <c r="J23" s="105"/>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B24" s="3" t="s">
@@ -4133,13 +4161,13 @@
       <c r="E24" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="F24" s="110" t="s">
+      <c r="F24" s="105" t="s">
         <v>217</v>
       </c>
-      <c r="G24" s="110"/>
-      <c r="H24" s="110"/>
-      <c r="I24" s="110"/>
-      <c r="J24" s="110"/>
+      <c r="G24" s="105"/>
+      <c r="H24" s="105"/>
+      <c r="I24" s="105"/>
+      <c r="J24" s="105"/>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B25" s="3" t="s">
@@ -4154,13 +4182,13 @@
       <c r="E25" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="F25" s="110" t="s">
+      <c r="F25" s="105" t="s">
         <v>218</v>
       </c>
-      <c r="G25" s="110"/>
-      <c r="H25" s="110"/>
-      <c r="I25" s="110"/>
-      <c r="J25" s="110"/>
+      <c r="G25" s="105"/>
+      <c r="H25" s="105"/>
+      <c r="I25" s="105"/>
+      <c r="J25" s="105"/>
       <c r="L25" s="101" t="s">
         <v>221</v>
       </c>
@@ -4190,13 +4218,13 @@
       <c r="E26" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="F26" s="110" t="s">
+      <c r="F26" s="105" t="s">
         <v>220</v>
       </c>
-      <c r="G26" s="110"/>
-      <c r="H26" s="110"/>
-      <c r="I26" s="110"/>
-      <c r="J26" s="110"/>
+      <c r="G26" s="105"/>
+      <c r="H26" s="105"/>
+      <c r="I26" s="105"/>
+      <c r="J26" s="105"/>
       <c r="L26" s="6">
         <v>800</v>
       </c>
@@ -4205,165 +4233,170 @@
         <v>25.006105006105006</v>
       </c>
       <c r="N26" s="6">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="O26" s="104">
-        <f>N26/16383</f>
-        <v>1.2207776353537203E-3</v>
+        <f>N26/4095</f>
+        <v>1.221001221001221E-3</v>
       </c>
       <c r="P26" s="103">
         <f>M26*O26</f>
-        <v>3.0526893738759699E-2</v>
+        <v>3.0532484744938956E-2</v>
       </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B27" s="102" t="s">
+      <c r="B27" s="132" t="s">
+        <v>225</v>
+      </c>
+      <c r="C27" s="132" t="s">
         <v>226</v>
       </c>
-      <c r="C27" s="102" t="s">
+      <c r="D27" s="132" t="s">
+        <v>5</v>
+      </c>
+      <c r="E27" s="132" t="s">
         <v>227</v>
       </c>
-      <c r="D27" s="102" t="s">
+      <c r="F27" s="133" t="s">
+        <v>229</v>
+      </c>
+      <c r="G27" s="133"/>
+      <c r="H27" s="133"/>
+      <c r="I27" s="133"/>
+      <c r="J27" s="133"/>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.45">
+      <c r="B28" s="102" t="s">
+        <v>230</v>
+      </c>
+      <c r="C28" s="102" t="s">
+        <v>231</v>
+      </c>
+      <c r="D28" s="102" t="s">
         <v>5</v>
       </c>
-      <c r="E27" s="102" t="s">
-        <v>228</v>
-      </c>
-      <c r="F27" s="112" t="s">
-        <v>230</v>
-      </c>
-      <c r="G27" s="112"/>
-      <c r="H27" s="112"/>
-      <c r="I27" s="112"/>
-      <c r="J27" s="112"/>
-    </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B30" s="5" t="s">
+      <c r="E28" s="102" t="s">
+        <v>232</v>
+      </c>
+      <c r="F28" s="129" t="s">
+        <v>233</v>
+      </c>
+      <c r="G28" s="130"/>
+      <c r="H28" s="130"/>
+      <c r="I28" s="130"/>
+      <c r="J28" s="131"/>
+    </row>
+    <row r="29" spans="2:16" x14ac:dyDescent="0.45">
+      <c r="O29" s="128"/>
+    </row>
+    <row r="31" spans="2:16" x14ac:dyDescent="0.45">
+      <c r="B31" s="5" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="31" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B31" s="7" t="s">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.45">
+      <c r="B32" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C31" s="9"/>
-      <c r="D31" s="7" t="s">
+      <c r="C32" s="9"/>
+      <c r="D32" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="E31" s="10"/>
-      <c r="F31" s="111" t="s">
+      <c r="E32" s="10"/>
+      <c r="F32" s="107" t="s">
         <v>47</v>
       </c>
-      <c r="G31" s="111"/>
-      <c r="H31" s="111"/>
-      <c r="I31" s="111"/>
-      <c r="J31" s="111"/>
-      <c r="K31" s="111"/>
-      <c r="L31" s="111"/>
-      <c r="M31" s="111"/>
-    </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B32" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>46</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="E32" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="F32" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="G32" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="H32" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="I32" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="J32" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="K32" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="L32" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="M32" s="16" t="s">
-        <v>121</v>
-      </c>
+      <c r="G32" s="107"/>
+      <c r="H32" s="107"/>
+      <c r="I32" s="107"/>
+      <c r="J32" s="107"/>
+      <c r="K32" s="107"/>
+      <c r="L32" s="107"/>
+      <c r="M32" s="107"/>
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B33" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>46</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E33" s="17"/>
-      <c r="F33" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="G33" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="H33" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="I33" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="J33" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="K33" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="L33" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="M33" s="21" t="s">
-        <v>122</v>
+        <v>36</v>
+      </c>
+      <c r="E33" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="G33" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="H33" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="I33" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="J33" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="K33" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B34" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>46</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="E34" s="9"/>
-      <c r="F34" s="9"/>
-      <c r="G34" s="9"/>
-      <c r="H34" s="9"/>
-      <c r="I34" s="9"/>
-      <c r="J34" s="9"/>
-      <c r="K34" s="9"/>
-      <c r="L34" s="9"/>
+        <v>37</v>
+      </c>
+      <c r="E34" s="17"/>
+      <c r="F34" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="G34" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="H34" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="I34" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="J34" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="K34" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="L34" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="M34" s="21" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B35" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>46</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
@@ -4376,13 +4409,13 @@
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B36" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>46</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
@@ -4395,11 +4428,13 @@
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B37" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C37" s="11"/>
+        <v>29</v>
+      </c>
+      <c r="C37" s="11" t="s">
+        <v>46</v>
+      </c>
       <c r="D37" s="8" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="E37" s="9"/>
       <c r="F37" s="9"/>
@@ -4412,13 +4447,11 @@
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B38" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C38" s="11" t="s">
-        <v>46</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="C38" s="11"/>
       <c r="D38" s="8" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E38" s="9"/>
       <c r="F38" s="9"/>
@@ -4431,13 +4464,13 @@
     </row>
     <row r="39" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B39" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>46</v>
       </c>
       <c r="D39" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E39" s="9"/>
       <c r="F39" s="9"/>
@@ -4450,13 +4483,13 @@
     </row>
     <row r="40" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B40" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>46</v>
       </c>
       <c r="D40" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E40" s="9"/>
       <c r="F40" s="9"/>
@@ -4469,13 +4502,13 @@
     </row>
     <row r="41" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B41" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>46</v>
       </c>
       <c r="D41" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E41" s="9"/>
       <c r="F41" s="9"/>
@@ -4488,13 +4521,13 @@
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B42" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C42" s="11" t="s">
         <v>46</v>
       </c>
       <c r="D42" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E42" s="9"/>
       <c r="F42" s="9"/>
@@ -4505,31 +4538,55 @@
       <c r="K42" s="9"/>
       <c r="L42" s="9"/>
     </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B45" s="5" t="s">
+    <row r="43" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B43" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C43" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+      <c r="I43" s="9"/>
+      <c r="J43" s="9"/>
+      <c r="K43" s="9"/>
+      <c r="L43" s="9"/>
+    </row>
+    <row r="46" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B46" s="5" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B46" s="6" t="s">
+    <row r="47" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B47" s="6" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="78" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B78" s="6" t="s">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B79" s="6" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.45">
-      <c r="B110" s="6" t="s">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B111" s="6" t="s">
         <v>201</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="E9:J9"/>
+    <mergeCell ref="E11:J11"/>
+    <mergeCell ref="E13:J13"/>
+    <mergeCell ref="F17:J17"/>
     <mergeCell ref="F25:J25"/>
     <mergeCell ref="E7:J7"/>
-    <mergeCell ref="F31:M31"/>
+    <mergeCell ref="F32:M32"/>
     <mergeCell ref="E8:J8"/>
     <mergeCell ref="E10:J10"/>
     <mergeCell ref="E12:J12"/>
@@ -4542,11 +4599,7 @@
     <mergeCell ref="F20:J20"/>
     <mergeCell ref="F26:J26"/>
     <mergeCell ref="F27:J27"/>
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="E9:J9"/>
-    <mergeCell ref="E11:J11"/>
-    <mergeCell ref="E13:J13"/>
-    <mergeCell ref="F17:J17"/>
+    <mergeCell ref="F28:J28"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4566,28 +4619,28 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="113" t="s">
+      <c r="B2" s="112" t="s">
         <v>105</v>
       </c>
-      <c r="D2" s="111" t="s">
+      <c r="D2" s="107" t="s">
         <v>84</v>
       </c>
-      <c r="E2" s="111" t="s">
+      <c r="E2" s="107" t="s">
         <v>72</v>
       </c>
-      <c r="F2" s="111"/>
-      <c r="G2" s="111"/>
-      <c r="H2" s="111"/>
-      <c r="I2" s="111" t="s">
+      <c r="F2" s="107"/>
+      <c r="G2" s="107"/>
+      <c r="H2" s="107"/>
+      <c r="I2" s="107" t="s">
         <v>71</v>
       </c>
-      <c r="J2" s="111"/>
-      <c r="K2" s="111"/>
-      <c r="L2" s="111"/>
+      <c r="J2" s="107"/>
+      <c r="K2" s="107"/>
+      <c r="L2" s="107"/>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B3" s="114"/>
-      <c r="D3" s="111"/>
+      <c r="B3" s="113"/>
+      <c r="D3" s="107"/>
       <c r="E3" s="7" t="s">
         <v>112</v>
       </c>
@@ -5769,35 +5822,35 @@
       </c>
     </row>
     <row r="3" spans="2:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="118" t="s">
+      <c r="B3" s="117" t="s">
         <v>169</v>
       </c>
-      <c r="C3" s="121" t="s">
+      <c r="C3" s="120" t="s">
         <v>171</v>
       </c>
-      <c r="D3" s="123" t="s">
+      <c r="D3" s="121" t="s">
         <v>172</v>
       </c>
-      <c r="F3" s="118" t="s">
+      <c r="F3" s="117" t="s">
         <v>72</v>
       </c>
-      <c r="G3" s="121"/>
-      <c r="H3" s="121"/>
-      <c r="I3" s="121"/>
-      <c r="J3" s="121" t="s">
+      <c r="G3" s="120"/>
+      <c r="H3" s="120"/>
+      <c r="I3" s="120"/>
+      <c r="J3" s="120" t="s">
         <v>71</v>
       </c>
-      <c r="K3" s="121"/>
-      <c r="L3" s="121"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="115" t="s">
+      <c r="K3" s="120"/>
+      <c r="L3" s="120"/>
+      <c r="M3" s="124"/>
+      <c r="N3" s="114" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.45">
-      <c r="B4" s="119"/>
-      <c r="C4" s="111"/>
-      <c r="D4" s="124"/>
+      <c r="B4" s="118"/>
+      <c r="C4" s="107"/>
+      <c r="D4" s="122"/>
       <c r="F4" s="60" t="s">
         <v>112</v>
       </c>
@@ -5822,12 +5875,12 @@
       <c r="M4" s="72" t="s">
         <v>115</v>
       </c>
-      <c r="N4" s="116"/>
+      <c r="N4" s="115"/>
     </row>
     <row r="5" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B5" s="120"/>
-      <c r="C5" s="122"/>
-      <c r="D5" s="125"/>
+      <c r="B5" s="125"/>
+      <c r="C5" s="126"/>
+      <c r="D5" s="127"/>
       <c r="F5" s="70">
         <v>1</v>
       </c>
@@ -5859,7 +5912,7 @@
         <f t="shared" si="0"/>
         <v>141</v>
       </c>
-      <c r="N5" s="117"/>
+      <c r="N5" s="116"/>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B6" s="66">
@@ -6247,35 +6300,35 @@
       </c>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.45">
-      <c r="B19" s="118" t="s">
+      <c r="B19" s="117" t="s">
         <v>169</v>
       </c>
-      <c r="C19" s="121" t="s">
+      <c r="C19" s="120" t="s">
         <v>171</v>
       </c>
-      <c r="D19" s="123" t="s">
+      <c r="D19" s="121" t="s">
         <v>172</v>
       </c>
-      <c r="F19" s="118" t="s">
+      <c r="F19" s="117" t="s">
         <v>72</v>
       </c>
-      <c r="G19" s="121"/>
-      <c r="H19" s="121"/>
-      <c r="I19" s="121"/>
-      <c r="J19" s="121" t="s">
+      <c r="G19" s="120"/>
+      <c r="H19" s="120"/>
+      <c r="I19" s="120"/>
+      <c r="J19" s="120" t="s">
         <v>71</v>
       </c>
-      <c r="K19" s="121"/>
-      <c r="L19" s="121"/>
-      <c r="M19" s="126"/>
-      <c r="N19" s="115" t="s">
+      <c r="K19" s="120"/>
+      <c r="L19" s="120"/>
+      <c r="M19" s="124"/>
+      <c r="N19" s="114" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.45">
-      <c r="B20" s="119"/>
-      <c r="C20" s="111"/>
-      <c r="D20" s="124"/>
+      <c r="B20" s="118"/>
+      <c r="C20" s="107"/>
+      <c r="D20" s="122"/>
       <c r="F20" s="60" t="s">
         <v>112</v>
       </c>
@@ -6300,12 +6353,12 @@
       <c r="M20" s="72" t="s">
         <v>115</v>
       </c>
-      <c r="N20" s="116"/>
+      <c r="N20" s="115"/>
     </row>
     <row r="21" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B21" s="127"/>
-      <c r="C21" s="113"/>
-      <c r="D21" s="128"/>
+      <c r="B21" s="119"/>
+      <c r="C21" s="112"/>
+      <c r="D21" s="123"/>
       <c r="F21" s="90">
         <v>12</v>
       </c>
@@ -6337,7 +6390,7 @@
         <f t="shared" ref="M21" si="7">L21+20</f>
         <v>152</v>
       </c>
-      <c r="N21" s="117"/>
+      <c r="N21" s="116"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B22" s="85">
@@ -6835,18 +6888,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="N3:N5"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="J3:M3"/>
     <mergeCell ref="N19:N21"/>
     <mergeCell ref="B19:B21"/>
     <mergeCell ref="C19:C21"/>
     <mergeCell ref="D19:D21"/>
     <mergeCell ref="F19:I19"/>
     <mergeCell ref="J19:M19"/>
-    <mergeCell ref="N3:N5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="C3:C5"/>
-    <mergeCell ref="D3:D5"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="J3:M3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>